<commit_message>
Updated JPN_grids model - 2025-09-17 10:13
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/Sets-vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{03DB9A9B-B2BC-4A17-AF2C-663C4A1A40BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E4ECF691-E777-449F-BB4E-A846300CB9C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4043" yWindow="4043" windowWidth="21599" windowHeight="12682" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VEDA_Sets-Comm" sheetId="2" r:id="rId1"/>
@@ -7823,7 +7823,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C07D208-0F09-4D70-80C9-1FC654D0DF43}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD9B02F1-5E4A-4686-9910-DE48A2D80F82}">
   <dimension ref="B9:E1116"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-21 00:24
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9224B8DD-5415-4AE7-A2C2-6CF76D2D98E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{13A5E855-24A4-45D0-B3FD-72B64D449F8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2915,7 +2915,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C288D49D-DED4-490A-8C9B-5549EBFB5EA8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4527BF12-B4D8-4E8D-819C-621210D40241}">
   <dimension ref="B9:E298"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-22 23:41
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5FAF3EEA-A8C1-4D7F-BE5E-FA3EDCB0940C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0EFF6C63-6144-4FD2-94F5-925D9A5EA906}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2915,7 +2915,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FC8B08A-413B-4F49-AC50-37C05DCA9584}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B523D178-9A8D-4020-8D93-07E8F3237E81}">
   <dimension ref="B9:E298"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-26 22:01
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{84DDB6FC-277D-4E2D-AFF0-CD18A8EA902A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8ABA0AC2-7DBF-4E03-BFFA-26B30BA4C4AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1272" uniqueCount="680">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1268" uniqueCount="678">
   <si>
     <t>~TFM_Psets</t>
   </si>
@@ -1622,12 +1622,6 @@
   </si>
   <si>
     <t>elc_spv_030</t>
-  </si>
-  <si>
-    <t>rez_spv_031</t>
-  </si>
-  <si>
-    <t>elc_spv_031</t>
   </si>
   <si>
     <t>rez_won_001</t>
@@ -2915,8 +2909,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6BD2A7E-4D35-4418-986F-91F08A39D4BB}">
-  <dimension ref="B9:E298"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC2D81D7-BAC6-45AE-AF77-6B02CB59D0EC}">
+  <dimension ref="B9:E297"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="9" spans="2:5" x14ac:dyDescent="0.45">
@@ -6953,20 +6947,6 @@
         <v>677</v>
       </c>
       <c r="E297" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="298" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B298" t="s">
-        <v>678</v>
-      </c>
-      <c r="C298" t="s">
-        <v>679</v>
-      </c>
-      <c r="D298" t="s">
-        <v>679</v>
-      </c>
-      <c r="E298" t="s">
         <v>105</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-27 10:13
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8ABA0AC2-7DBF-4E03-BFFA-26B30BA4C4AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CE00B708-ECE7-4322-B8A6-032F3708F868}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2909,7 +2909,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC2D81D7-BAC6-45AE-AF77-6B02CB59D0EC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{010EA616-D442-4756-B5B3-E4180AD7F7A1}">
   <dimension ref="B9:E297"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-27 20:57
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CE00B708-ECE7-4322-B8A6-032F3708F868}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{83BEB3DC-ED77-4EEE-9F37-B42488D9C5E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2909,7 +2909,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{010EA616-D442-4756-B5B3-E4180AD7F7A1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C8C131D-7922-4392-B0D4-460BD1E615F9}">
   <dimension ref="B9:E297"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>